<commit_message>
Aktualizovat Klice_Teplo.xlsx - oprava Jednotek=1 pro TSJUSTDANCE/T_PAUS
Uzivatel opravil zdrojova data (puvodne Jednotek=0 = neuctovalo se,
i kdyz mel byt pausal aktivni).
</commit_message>
<xml_diff>
--- a/core/management/commands/Klice_Teplo.xlsx
+++ b/core/management/commands/Klice_Teplo.xlsx
@@ -5,16 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/daniel/Desktop/RenteX/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{37A3361A-C5A0-3441-A7BA-37DD46D98785}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F0E9B83-3623-734F-8DC7-4D3B1B7CCF5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2980" yWindow="2180" windowWidth="28240" windowHeight="17240" xr2:uid="{815A4C60-1CF7-594C-87A9-725B82D83013}"/>
+    <workbookView xWindow="9260" yWindow="1320" windowWidth="28240" windowHeight="17240" xr2:uid="{815A4C60-1CF7-594C-87A9-725B82D83013}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">List1!$A$1:$M$78</definedName>
+  </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -778,8 +781,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23C877DC-9AC4-1942-9E65-205082DDFCCE}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="30.5" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -822,7 +829,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>13</v>
       </c>
@@ -861,7 +868,7 @@
       </c>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>13</v>
       </c>
@@ -900,7 +907,7 @@
       </c>
       <c r="M3" s="2"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>13</v>
       </c>
@@ -939,7 +946,7 @@
       </c>
       <c r="M4" s="2"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
@@ -978,7 +985,7 @@
       </c>
       <c r="M5" s="2"/>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" s="2" t="s">
         <v>20</v>
       </c>
@@ -1034,7 +1041,7 @@
         <v>27</v>
       </c>
       <c r="F7" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G7" s="3">
         <v>1</v>
@@ -1056,7 +1063,7 @@
       </c>
       <c r="M7" s="2"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" s="2" t="s">
         <v>24</v>
       </c>
@@ -1095,7 +1102,7 @@
       </c>
       <c r="M8" s="2"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" s="2" t="s">
         <v>24</v>
       </c>
@@ -1134,7 +1141,7 @@
       </c>
       <c r="M9" s="2"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>29</v>
       </c>
@@ -1175,7 +1182,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
@@ -1216,7 +1223,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" s="2" t="s">
         <v>33</v>
       </c>
@@ -1255,7 +1262,7 @@
       </c>
       <c r="M12" s="2"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
@@ -1294,7 +1301,7 @@
       </c>
       <c r="M13" s="2"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>35</v>
       </c>
@@ -1333,7 +1340,7 @@
       </c>
       <c r="M14" s="2"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" s="2" t="s">
         <v>35</v>
       </c>
@@ -1411,7 +1418,7 @@
       </c>
       <c r="M16" s="2"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" s="2" t="s">
         <v>39</v>
       </c>
@@ -1489,7 +1496,7 @@
       </c>
       <c r="M18" s="2"/>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" s="2" t="s">
         <v>41</v>
       </c>
@@ -1528,7 +1535,7 @@
       </c>
       <c r="M19" s="2"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" s="2" t="s">
         <v>45</v>
       </c>
@@ -1567,7 +1574,7 @@
       </c>
       <c r="M20" s="2"/>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" s="2" t="s">
         <v>45</v>
       </c>
@@ -1606,7 +1613,7 @@
       </c>
       <c r="M21" s="2"/>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" s="2" t="s">
         <v>48</v>
       </c>
@@ -1645,7 +1652,7 @@
       </c>
       <c r="M22" s="2"/>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" s="2" t="s">
         <v>48</v>
       </c>
@@ -1684,7 +1691,7 @@
       </c>
       <c r="M23" s="2"/>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" s="2" t="s">
         <v>48</v>
       </c>
@@ -1723,7 +1730,7 @@
       </c>
       <c r="M24" s="2"/>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" s="2" t="s">
         <v>52</v>
       </c>
@@ -1762,7 +1769,7 @@
       </c>
       <c r="M25" s="2"/>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" s="2" t="s">
         <v>52</v>
       </c>
@@ -1801,7 +1808,7 @@
       </c>
       <c r="M26" s="2"/>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" s="2" t="s">
         <v>56</v>
       </c>
@@ -1840,7 +1847,7 @@
       </c>
       <c r="M27" s="2"/>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" s="2" t="s">
         <v>56</v>
       </c>
@@ -1879,7 +1886,7 @@
       </c>
       <c r="M28" s="2"/>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A29" s="2" t="s">
         <v>56</v>
       </c>
@@ -1918,7 +1925,7 @@
       </c>
       <c r="M29" s="2"/>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" s="2" t="s">
         <v>56</v>
       </c>
@@ -1996,7 +2003,7 @@
       </c>
       <c r="M31" s="2"/>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" s="2" t="s">
         <v>61</v>
       </c>
@@ -2035,7 +2042,7 @@
       </c>
       <c r="M32" s="2"/>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" s="2" t="s">
         <v>64</v>
       </c>
@@ -2074,7 +2081,7 @@
       </c>
       <c r="M33" s="2"/>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" s="2" t="s">
         <v>64</v>
       </c>
@@ -2113,7 +2120,7 @@
       </c>
       <c r="M34" s="2"/>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" s="2" t="s">
         <v>64</v>
       </c>
@@ -2152,7 +2159,7 @@
       </c>
       <c r="M35" s="2"/>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" s="2" t="s">
         <v>64</v>
       </c>
@@ -2193,7 +2200,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" s="2" t="s">
         <v>64</v>
       </c>
@@ -2232,7 +2239,7 @@
       </c>
       <c r="M37" s="2"/>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" s="2" t="s">
         <v>70</v>
       </c>
@@ -2271,7 +2278,7 @@
       </c>
       <c r="M38" s="2"/>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" s="2" t="s">
         <v>70</v>
       </c>
@@ -2310,7 +2317,7 @@
       </c>
       <c r="M39" s="2"/>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" s="2" t="s">
         <v>74</v>
       </c>
@@ -2349,7 +2356,7 @@
       </c>
       <c r="M40" s="2"/>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" s="2" t="s">
         <v>76</v>
       </c>
@@ -2427,7 +2434,7 @@
       </c>
       <c r="M42" s="2"/>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" s="2" t="s">
         <v>79</v>
       </c>
@@ -2466,7 +2473,7 @@
       </c>
       <c r="M43" s="2"/>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" s="2" t="s">
         <v>79</v>
       </c>
@@ -2505,7 +2512,7 @@
       </c>
       <c r="M44" s="2"/>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" s="2" t="s">
         <v>79</v>
       </c>
@@ -2544,7 +2551,7 @@
       </c>
       <c r="M45" s="2"/>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" s="2" t="s">
         <v>79</v>
       </c>
@@ -2583,7 +2590,7 @@
       </c>
       <c r="M46" s="2"/>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" s="2" t="s">
         <v>84</v>
       </c>
@@ -2622,7 +2629,7 @@
       </c>
       <c r="M47" s="2"/>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" s="2" t="s">
         <v>84</v>
       </c>
@@ -2661,7 +2668,7 @@
       </c>
       <c r="M48" s="2"/>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" s="2" t="s">
         <v>87</v>
       </c>
@@ -2700,7 +2707,7 @@
       </c>
       <c r="M49" s="2"/>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" s="2" t="s">
         <v>87</v>
       </c>
@@ -2739,7 +2746,7 @@
       </c>
       <c r="M50" s="2"/>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A51" s="2" t="s">
         <v>87</v>
       </c>
@@ -2778,7 +2785,7 @@
       </c>
       <c r="M51" s="2"/>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" s="2" t="s">
         <v>87</v>
       </c>
@@ -2817,7 +2824,7 @@
       </c>
       <c r="M52" s="2"/>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" s="2" t="s">
         <v>87</v>
       </c>
@@ -2856,7 +2863,7 @@
       </c>
       <c r="M53" s="2"/>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" s="2" t="s">
         <v>93</v>
       </c>
@@ -2895,7 +2902,7 @@
       </c>
       <c r="M54" s="2"/>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" s="2" t="s">
         <v>93</v>
       </c>
@@ -2934,7 +2941,7 @@
       </c>
       <c r="M55" s="2"/>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" s="2" t="s">
         <v>93</v>
       </c>
@@ -2973,7 +2980,7 @@
       </c>
       <c r="M56" s="2"/>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A57" s="2" t="s">
         <v>97</v>
       </c>
@@ -3012,7 +3019,7 @@
       </c>
       <c r="M57" s="2"/>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" s="2" t="s">
         <v>97</v>
       </c>
@@ -3051,7 +3058,7 @@
       </c>
       <c r="M58" s="2"/>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" s="2" t="s">
         <v>97</v>
       </c>
@@ -3090,7 +3097,7 @@
       </c>
       <c r="M59" s="2"/>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" s="2" t="s">
         <v>97</v>
       </c>
@@ -3129,7 +3136,7 @@
       </c>
       <c r="M60" s="2"/>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" s="2" t="s">
         <v>102</v>
       </c>
@@ -3168,7 +3175,7 @@
       </c>
       <c r="M61" s="2"/>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A62" s="2" t="s">
         <v>102</v>
       </c>
@@ -3207,7 +3214,7 @@
       </c>
       <c r="M62" s="2"/>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A63" s="2" t="s">
         <v>104</v>
       </c>
@@ -3246,7 +3253,7 @@
       </c>
       <c r="M63" s="2"/>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" s="2" t="s">
         <v>104</v>
       </c>
@@ -3285,7 +3292,7 @@
       </c>
       <c r="M64" s="2"/>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" s="2" t="s">
         <v>104</v>
       </c>
@@ -3324,7 +3331,7 @@
       </c>
       <c r="M65" s="2"/>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" s="2" t="s">
         <v>104</v>
       </c>
@@ -3363,7 +3370,7 @@
       </c>
       <c r="M66" s="2"/>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" s="2" t="s">
         <v>104</v>
       </c>
@@ -3402,7 +3409,7 @@
       </c>
       <c r="M67" s="2"/>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" s="2" t="s">
         <v>104</v>
       </c>
@@ -3441,7 +3448,7 @@
       </c>
       <c r="M68" s="2"/>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" s="2" t="s">
         <v>104</v>
       </c>
@@ -3480,7 +3487,7 @@
       </c>
       <c r="M69" s="2"/>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" s="2" t="s">
         <v>104</v>
       </c>
@@ -3519,7 +3526,7 @@
       </c>
       <c r="M70" s="2"/>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" s="2" t="s">
         <v>104</v>
       </c>
@@ -3558,7 +3565,7 @@
       </c>
       <c r="M71" s="2"/>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" s="2" t="s">
         <v>104</v>
       </c>
@@ -3597,7 +3604,7 @@
       </c>
       <c r="M72" s="2"/>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A73" s="2" t="s">
         <v>104</v>
       </c>
@@ -3636,7 +3643,7 @@
       </c>
       <c r="M73" s="2"/>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A74" s="2" t="s">
         <v>104</v>
       </c>
@@ -3677,7 +3684,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" s="2" t="s">
         <v>118</v>
       </c>
@@ -3716,7 +3723,7 @@
       </c>
       <c r="M75" s="2"/>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" s="2" t="s">
         <v>118</v>
       </c>
@@ -3755,7 +3762,7 @@
       </c>
       <c r="M76" s="2"/>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" s="2" t="s">
         <v>121</v>
       </c>
@@ -3794,7 +3801,7 @@
       </c>
       <c r="M77" s="2"/>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:13" hidden="1" x14ac:dyDescent="0.2">
       <c r="A78" s="2" t="s">
         <v>121</v>
       </c>
@@ -3834,6 +3841,13 @@
       <c r="M78" s="2"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:M78" xr:uid="{23C877DC-9AC4-1942-9E65-205082DDFCCE}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="T_PAUS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>